<commit_message>
Daily Activity Tracker Day 2
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15511D1E-8ECC-4DD0-A2B3-417A7D7CA5C0}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3231E24-2F97-4BBA-8506-FEE00971A34F}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="59">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -208,6 +208,15 @@
   </si>
   <si>
     <t>Attended all class and bit tired after evening class.</t>
+  </si>
+  <si>
+    <t>Good</t>
+  </si>
+  <si>
+    <t>Satisfied</t>
+  </si>
+  <si>
+    <t>Feeling good today</t>
   </si>
 </sst>
 </file>
@@ -1032,29 +1041,53 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="15" t="str">
+    <row r="7" spans="1:14" ht="15">
+      <c r="A7" s="13">
+        <v>46247</v>
+      </c>
+      <c r="B7" s="14">
+        <v>540</v>
+      </c>
+      <c r="C7" s="14">
+        <v>20</v>
+      </c>
+      <c r="D7" s="14">
+        <v>30</v>
+      </c>
+      <c r="E7" s="14">
+        <v>30</v>
+      </c>
+      <c r="F7" s="14">
+        <v>150</v>
+      </c>
+      <c r="G7" s="14">
+        <v>3</v>
+      </c>
+      <c r="H7" s="14">
+        <v>60</v>
+      </c>
+      <c r="I7" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J7" s="15" t="str">
+        <v>830</v>
+      </c>
+      <c r="J7" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="17"/>
-    </row>
-    <row r="8" spans="1:14">
+        <v>610</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="15">
       <c r="A8" s="13"/>
       <c r="B8" s="14"/>
       <c r="C8" s="14"/>
@@ -1074,7 +1107,9 @@
       <c r="K8" s="16"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
-      <c r="N8" s="17"/>
+      <c r="N8" s="17" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker Day 3
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3231E24-2F97-4BBA-8506-FEE00971A34F}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DCAD361-2B8A-4E15-B025-BCA941A458B3}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -217,6 +217,9 @@
   </si>
   <si>
     <t>Feeling good today</t>
+  </si>
+  <si>
+    <t>High</t>
   </si>
 </sst>
 </file>
@@ -1088,28 +1091,48 @@
       </c>
     </row>
     <row r="8" spans="1:14" ht="15">
-      <c r="A8" s="13"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="15" t="str">
+      <c r="A8" s="13">
+        <v>46248</v>
+      </c>
+      <c r="B8" s="14">
+        <v>520</v>
+      </c>
+      <c r="C8" s="14">
+        <v>15</v>
+      </c>
+      <c r="D8" s="14">
+        <v>60</v>
+      </c>
+      <c r="E8" s="14">
+        <v>60</v>
+      </c>
+      <c r="F8" s="14">
+        <v>250</v>
+      </c>
+      <c r="G8" s="14">
+        <v>5</v>
+      </c>
+      <c r="H8" s="14">
+        <v>30</v>
+      </c>
+      <c r="I8" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J8" s="15" t="str">
+        <v>935</v>
+      </c>
+      <c r="J8" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="17" t="s">
-        <v>58</v>
-      </c>
+        <v>505</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N8" s="17"/>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker Day 4
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DCAD361-2B8A-4E15-B025-BCA941A458B3}"/>
+  <xr:revisionPtr revIDLastSave="71" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81D9244A-F5AC-4E42-948F-4B5206D3F033}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="63">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -220,6 +220,15 @@
   </si>
   <si>
     <t>High</t>
+  </si>
+  <si>
+    <t>Good day</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>Had enough rest and high energy</t>
   </si>
 </sst>
 </file>
@@ -1132,31 +1141,57 @@
       <c r="M8" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="N8" s="17"/>
-    </row>
-    <row r="9" spans="1:14">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15" t="str">
+      <c r="N8" s="17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="30.75">
+      <c r="A9" s="13">
+        <v>46249</v>
+      </c>
+      <c r="B9" s="14">
+        <v>630</v>
+      </c>
+      <c r="C9" s="14">
+        <v>20</v>
+      </c>
+      <c r="D9" s="14">
+        <v>120</v>
+      </c>
+      <c r="E9" s="14">
+        <v>60</v>
+      </c>
+      <c r="F9" s="14">
+        <v>0</v>
+      </c>
+      <c r="G9" s="14">
+        <v>0</v>
+      </c>
+      <c r="H9" s="14">
+        <v>30</v>
+      </c>
+      <c r="I9" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J9" s="15" t="str">
+        <v>860</v>
+      </c>
+      <c r="J9" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="17"/>
-    </row>
-    <row r="10" spans="1:14">
+        <v>580</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="15">
       <c r="A10" s="13"/>
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>

</xml_diff>

<commit_message>
Daily Activity Tracker Day 6
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81D9244A-F5AC-4E42-948F-4B5206D3F033}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D998BDE0-10FE-4BAC-B92D-C38B8FDD8310}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="64">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -229,6 +229,9 @@
   </si>
   <si>
     <t>Had enough rest and high energy</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
   </si>
 </sst>
 </file>
@@ -1192,26 +1195,48 @@
       </c>
     </row>
     <row r="10" spans="1:14" ht="15">
-      <c r="A10" s="13"/>
+      <c r="A10" s="13">
+        <v>46250</v>
+      </c>
       <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="15" t="str">
+      <c r="C10" s="14">
+        <v>30</v>
+      </c>
+      <c r="D10" s="14">
+        <v>150</v>
+      </c>
+      <c r="E10" s="14">
+        <v>60</v>
+      </c>
+      <c r="F10" s="14">
+        <v>0</v>
+      </c>
+      <c r="G10" s="14">
+        <v>0</v>
+      </c>
+      <c r="H10" s="14">
+        <v>30</v>
+      </c>
+      <c r="I10" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J10" s="15" t="str">
+        <v>270</v>
+      </c>
+      <c r="J10" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
-      <c r="N10" s="17"/>
+        <v>1170</v>
+      </c>
+      <c r="K10" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L10" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N10" s="17" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker- 17Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="82" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D998BDE0-10FE-4BAC-B92D-C38B8FDD8310}"/>
+  <xr:revisionPtr revIDLastSave="98" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B000743E-5CEE-484A-9D01-38673BD9EE78}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="65">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -232,6 +232,9 @@
   </si>
   <si>
     <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>Had interactive session.</t>
   </si>
 </sst>
 </file>
@@ -1198,7 +1201,9 @@
       <c r="A10" s="13">
         <v>46250</v>
       </c>
-      <c r="B10" s="14"/>
+      <c r="B10" s="14">
+        <v>600</v>
+      </c>
       <c r="C10" s="14">
         <v>30</v>
       </c>
@@ -1219,11 +1224,11 @@
       </c>
       <c r="I10" s="15">
         <f t="shared" si="0"/>
-        <v>270</v>
+        <v>870</v>
       </c>
       <c r="J10" s="15">
         <f t="shared" si="1"/>
-        <v>1170</v>
+        <v>570</v>
       </c>
       <c r="K10" s="16" t="s">
         <v>61</v>
@@ -1238,29 +1243,53 @@
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
-      <c r="A11" s="13"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="15" t="str">
+    <row r="11" spans="1:14" ht="15">
+      <c r="A11" s="13">
+        <v>46251</v>
+      </c>
+      <c r="B11" s="14">
+        <v>530</v>
+      </c>
+      <c r="C11" s="14">
+        <v>30</v>
+      </c>
+      <c r="D11" s="14">
+        <v>120</v>
+      </c>
+      <c r="E11" s="14">
+        <v>60</v>
+      </c>
+      <c r="F11" s="14">
+        <v>350</v>
+      </c>
+      <c r="G11" s="14">
+        <v>7</v>
+      </c>
+      <c r="H11" s="14">
+        <v>30</v>
+      </c>
+      <c r="I11" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="15" t="str">
+        <v>1120</v>
+      </c>
+      <c r="J11" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="17"/>
-    </row>
-    <row r="12" spans="1:14">
+        <v>320</v>
+      </c>
+      <c r="K11" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="15">
       <c r="A12" s="13"/>
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 18Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="98" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B000743E-5CEE-484A-9D01-38673BD9EE78}"/>
+  <xr:revisionPtr revIDLastSave="110" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{092CEB32-0866-4F81-BC3E-3AE4964B00F9}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -235,6 +235,12 @@
   </si>
   <si>
     <t>Had interactive session.</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Not felt good today.</t>
   </si>
 </sst>
 </file>
@@ -1290,26 +1296,50 @@
       </c>
     </row>
     <row r="12" spans="1:14" ht="15">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+      <c r="A12" s="13">
+        <v>46252</v>
+      </c>
+      <c r="B12" s="14">
+        <v>620</v>
+      </c>
+      <c r="C12" s="14">
+        <v>30</v>
+      </c>
+      <c r="D12" s="14">
+        <v>150</v>
+      </c>
+      <c r="E12" s="14">
+        <v>60</v>
+      </c>
+      <c r="F12" s="14">
+        <v>200</v>
+      </c>
+      <c r="G12" s="14">
+        <v>4</v>
+      </c>
+      <c r="H12" s="14">
+        <v>30</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>1090</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="17"/>
+        <v>350</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 19 Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="110" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{092CEB32-0866-4F81-BC3E-3AE4964B00F9}"/>
+  <xr:revisionPtr revIDLastSave="126" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EA01C33-C36B-4170-9732-B0E568F50E7D}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -241,6 +241,9 @@
   </si>
   <si>
     <t>Not felt good today.</t>
+  </si>
+  <si>
+    <t>Had a good day.</t>
   </si>
 </sst>
 </file>
@@ -1341,27 +1344,51 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15" t="str">
+    <row r="13" spans="1:14" ht="15">
+      <c r="A13" s="13">
+        <v>46253</v>
+      </c>
+      <c r="B13" s="14">
+        <v>600</v>
+      </c>
+      <c r="C13" s="14">
+        <v>20</v>
+      </c>
+      <c r="D13" s="14">
+        <v>120</v>
+      </c>
+      <c r="E13" s="14">
+        <v>60</v>
+      </c>
+      <c r="F13" s="14">
+        <v>250</v>
+      </c>
+      <c r="G13" s="14">
+        <v>5</v>
+      </c>
+      <c r="H13" s="14">
+        <v>0</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="17"/>
+        <v>390</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 20Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30413"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="126" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EA01C33-C36B-4170-9732-B0E568F50E7D}"/>
+  <xr:revisionPtr revIDLastSave="138" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F2B36DB-E106-4D29-86D5-6344C7487FFC}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="69">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -244,6 +244,9 @@
   </si>
   <si>
     <t>Had a good day.</t>
+  </si>
+  <si>
+    <t>Completed all tasks.</t>
   </si>
 </sst>
 </file>
@@ -1390,27 +1393,51 @@
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+    <row r="14" spans="1:14" ht="15">
+      <c r="A14" s="13">
+        <v>46254</v>
+      </c>
+      <c r="B14" s="14">
+        <v>650</v>
+      </c>
+      <c r="C14" s="14">
+        <v>20</v>
+      </c>
+      <c r="D14" s="14">
+        <v>150</v>
+      </c>
+      <c r="E14" s="14">
+        <v>60</v>
+      </c>
+      <c r="F14" s="14">
+        <v>150</v>
+      </c>
+      <c r="G14" s="14">
+        <v>3</v>
+      </c>
+      <c r="H14" s="14">
+        <v>20</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="17"/>
+        <v>390</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 21Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="138" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F2B36DB-E106-4D29-86D5-6344C7487FFC}"/>
+  <xr:revisionPtr revIDLastSave="152" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B6960D6-AAEB-4662-8D63-200066D9C0FD}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="70">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -247,6 +247,9 @@
   </si>
   <si>
     <t>Completed all tasks.</t>
+  </si>
+  <si>
+    <t>Learned new concepts.</t>
   </si>
 </sst>
 </file>
@@ -1439,27 +1442,51 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
-      <c r="A15" s="13"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="str">
+    <row r="15" spans="1:14" ht="15">
+      <c r="A15" s="13">
+        <v>46255</v>
+      </c>
+      <c r="B15" s="14">
+        <v>650</v>
+      </c>
+      <c r="C15" s="14">
+        <v>20</v>
+      </c>
+      <c r="D15" s="14">
+        <v>90</v>
+      </c>
+      <c r="E15" s="14">
+        <v>120</v>
+      </c>
+      <c r="F15" s="14">
+        <v>50</v>
+      </c>
+      <c r="G15" s="14">
+        <v>1</v>
+      </c>
+      <c r="H15" s="14">
+        <v>30</v>
+      </c>
+      <c r="I15" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="15" t="str">
+        <v>960</v>
+      </c>
+      <c r="J15" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
-      <c r="N15" s="17"/>
+        <v>480</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N15" s="17" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 23Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="152" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B6960D6-AAEB-4662-8D63-200066D9C0FD}"/>
+  <xr:revisionPtr revIDLastSave="177" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80078BA2-9D08-4D86-B52E-D67A1BC9B57D}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="71">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -250,6 +250,9 @@
   </si>
   <si>
     <t>Learned new concepts.</t>
+  </si>
+  <si>
+    <t>Learned new things.</t>
   </si>
 </sst>
 </file>
@@ -1488,49 +1491,97 @@
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="str">
+    <row r="16" spans="1:14" ht="15">
+      <c r="A16" s="13">
+        <v>46256</v>
+      </c>
+      <c r="B16" s="14">
+        <v>600</v>
+      </c>
+      <c r="C16" s="14">
+        <v>30</v>
+      </c>
+      <c r="D16" s="14">
+        <v>180</v>
+      </c>
+      <c r="E16" s="14">
+        <v>120</v>
+      </c>
+      <c r="F16" s="14">
+        <v>0</v>
+      </c>
+      <c r="G16" s="14">
+        <v>0</v>
+      </c>
+      <c r="H16" s="14">
+        <v>20</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="17"/>
-    </row>
-    <row r="17" spans="1:14">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15" t="str">
+        <v>490</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N16" s="17" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="15">
+      <c r="A17" s="13">
+        <v>46257</v>
+      </c>
+      <c r="B17" s="14">
+        <v>630</v>
+      </c>
+      <c r="C17" s="14">
+        <v>20</v>
+      </c>
+      <c r="D17" s="14">
+        <v>150</v>
+      </c>
+      <c r="E17" s="14">
+        <v>90</v>
+      </c>
+      <c r="F17" s="14">
+        <v>0</v>
+      </c>
+      <c r="G17" s="14">
+        <v>0</v>
+      </c>
+      <c r="H17" s="14">
+        <v>20</v>
+      </c>
+      <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="15" t="str">
+        <v>910</v>
+      </c>
+      <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
-      <c r="N17" s="17"/>
+        <v>530</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 24Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="177" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80078BA2-9D08-4D86-B52E-D67A1BC9B57D}"/>
+  <xr:revisionPtr revIDLastSave="190" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39E9EA73-5D0F-42EC-9030-C75DE91D17F8}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="72">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -253,6 +253,9 @@
   </si>
   <si>
     <t>Learned new things.</t>
+  </si>
+  <si>
+    <t>Tired after all classes</t>
   </si>
 </sst>
 </file>
@@ -1583,27 +1586,51 @@
         <v>60</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+    <row r="18" spans="1:14" ht="15">
+      <c r="A18" s="13">
+        <v>46258</v>
+      </c>
+      <c r="B18" s="14">
+        <v>570</v>
+      </c>
+      <c r="C18" s="14">
+        <v>20</v>
+      </c>
+      <c r="D18" s="14">
+        <v>60</v>
+      </c>
+      <c r="E18" s="14">
+        <v>30</v>
+      </c>
+      <c r="F18" s="14">
+        <v>400</v>
+      </c>
+      <c r="G18" s="14">
+        <v>8</v>
+      </c>
+      <c r="H18" s="14">
+        <v>20</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>1100</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="17"/>
+        <v>340</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="13"/>

</xml_diff>

<commit_message>
Daily activity Tracker 25Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="190" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39E9EA73-5D0F-42EC-9030-C75DE91D17F8}"/>
+  <xr:revisionPtr revIDLastSave="204" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6121D40-4C86-478A-B1CF-DAB2F1331C62}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="73">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -256,6 +256,9 @@
   </si>
   <si>
     <t>Tired after all classes</t>
+  </si>
+  <si>
+    <t>Average day.</t>
   </si>
 </sst>
 </file>
@@ -1632,27 +1635,51 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+    <row r="19" spans="1:14" ht="15">
+      <c r="A19" s="13">
+        <v>46259</v>
+      </c>
+      <c r="B19" s="14">
+        <v>540</v>
+      </c>
+      <c r="C19" s="14">
+        <v>30</v>
+      </c>
+      <c r="D19" s="14">
+        <v>120</v>
+      </c>
+      <c r="E19" s="14">
+        <v>120</v>
+      </c>
+      <c r="F19" s="14">
+        <v>300</v>
+      </c>
+      <c r="G19" s="14">
+        <v>6</v>
+      </c>
+      <c r="H19" s="14">
+        <v>30</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>1140</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="17"/>
+        <v>300</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 26Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="204" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6121D40-4C86-478A-B1CF-DAB2F1331C62}"/>
+  <xr:revisionPtr revIDLastSave="216" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D4A959D-1701-469F-AC92-6C3C5EC20776}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="75">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -259,6 +259,12 @@
   </si>
   <si>
     <t>Average day.</t>
+  </si>
+  <si>
+    <t>Unsatisfied</t>
+  </si>
+  <si>
+    <t>Having fever and cold.</t>
   </si>
 </sst>
 </file>
@@ -1681,27 +1687,51 @@
         <v>72</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+    <row r="20" spans="1:14" ht="15">
+      <c r="A20" s="13">
+        <v>46260</v>
+      </c>
+      <c r="B20" s="14">
+        <v>580</v>
+      </c>
+      <c r="C20" s="14">
+        <v>30</v>
+      </c>
+      <c r="D20" s="14">
+        <v>60</v>
+      </c>
+      <c r="E20" s="14">
+        <v>60</v>
+      </c>
+      <c r="F20" s="14">
+        <v>300</v>
+      </c>
+      <c r="G20" s="14">
+        <v>6</v>
+      </c>
+      <c r="H20" s="14">
+        <v>0</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>1030</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="17"/>
+        <v>410</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 27Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="216" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D4A959D-1701-469F-AC92-6C3C5EC20776}"/>
+  <xr:revisionPtr revIDLastSave="228" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12A7B263-96B1-4D5E-B122-228E2152C826}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="75">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1733,27 +1733,51 @@
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+    <row r="21" spans="1:14" ht="15">
+      <c r="A21" s="13">
+        <v>46261</v>
+      </c>
+      <c r="B21" s="14">
+        <v>550</v>
+      </c>
+      <c r="C21" s="14">
+        <v>30</v>
+      </c>
+      <c r="D21" s="14">
+        <v>60</v>
+      </c>
+      <c r="E21" s="14">
+        <v>60</v>
+      </c>
+      <c r="F21" s="14">
+        <v>150</v>
+      </c>
+      <c r="G21" s="14">
+        <v>3</v>
+      </c>
+      <c r="H21" s="14">
+        <v>20</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>870</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
-      <c r="N21" s="17"/>
+        <v>570</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N21" s="17" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 28Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="228" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12A7B263-96B1-4D5E-B122-228E2152C826}"/>
+  <xr:revisionPtr revIDLastSave="240" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A23B4D2-FF62-45D0-BFAA-BCA2A2A431B6}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="76">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -265,6 +265,9 @@
   </si>
   <si>
     <t>Having fever and cold.</t>
+  </si>
+  <si>
+    <t>Learned new topics.</t>
   </si>
 </sst>
 </file>
@@ -1779,27 +1782,51 @@
         <v>60</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+    <row r="22" spans="1:14" ht="15">
+      <c r="A22" s="13">
+        <v>46262</v>
+      </c>
+      <c r="B22" s="14">
+        <v>570</v>
+      </c>
+      <c r="C22" s="14">
+        <v>30</v>
+      </c>
+      <c r="D22" s="14">
+        <v>120</v>
+      </c>
+      <c r="E22" s="14">
+        <v>120</v>
+      </c>
+      <c r="F22" s="14">
+        <v>100</v>
+      </c>
+      <c r="G22" s="14">
+        <v>2</v>
+      </c>
+      <c r="H22" s="14">
+        <v>0</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>940</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="17"/>
+        <v>500</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 29Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="240" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A23B4D2-FF62-45D0-BFAA-BCA2A2A431B6}"/>
+  <xr:revisionPtr revIDLastSave="254" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F82C8F12-DA17-49C3-8FAB-F13C10240A0D}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="76">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1828,27 +1828,51 @@
         <v>75</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+    <row r="23" spans="1:14" ht="15">
+      <c r="A23" s="13">
+        <v>46263</v>
+      </c>
+      <c r="B23" s="14">
+        <v>550</v>
+      </c>
+      <c r="C23" s="14">
+        <v>30</v>
+      </c>
+      <c r="D23" s="14">
+        <v>120</v>
+      </c>
+      <c r="E23" s="14">
+        <v>120</v>
+      </c>
+      <c r="F23" s="14">
+        <v>50</v>
+      </c>
+      <c r="G23" s="14">
+        <v>1</v>
+      </c>
+      <c r="H23" s="14">
+        <v>30</v>
+      </c>
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>900</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
-      <c r="N23" s="17"/>
+        <v>540</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N23" s="17" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="24" spans="1:14">
       <c r="A24" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 30Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="254" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F82C8F12-DA17-49C3-8FAB-F13C10240A0D}"/>
+  <xr:revisionPtr revIDLastSave="268" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C2A96FB-EBCA-4949-BAF0-49353C6B1C5B}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="77">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -268,6 +268,9 @@
   </si>
   <si>
     <t>Learned new topics.</t>
+  </si>
+  <si>
+    <t>Had enough rest</t>
   </si>
 </sst>
 </file>
@@ -1874,27 +1877,51 @@
         <v>68</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="15" t="str">
+    <row r="24" spans="1:14" ht="15">
+      <c r="A24" s="13">
+        <v>46264</v>
+      </c>
+      <c r="B24" s="14">
+        <v>600</v>
+      </c>
+      <c r="C24" s="14">
+        <v>45</v>
+      </c>
+      <c r="D24" s="14">
+        <v>120</v>
+      </c>
+      <c r="E24" s="14">
+        <v>60</v>
+      </c>
+      <c r="F24" s="14">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14">
+        <v>0</v>
+      </c>
+      <c r="H24" s="14">
+        <v>20</v>
+      </c>
+      <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
+        <v>845</v>
+      </c>
+      <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="17"/>
+        <v>595</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N24" s="17" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="25" spans="1:14">
       <c r="A25" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 31Aug
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="268" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C2A96FB-EBCA-4949-BAF0-49353C6B1C5B}"/>
+  <xr:revisionPtr revIDLastSave="280" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{402A95FB-9466-4BD5-B9A3-5E0C9D13C9E1}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="78">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -271,6 +271,9 @@
   </si>
   <si>
     <t>Had enough rest</t>
+  </si>
+  <si>
+    <t>Attended workshop done by google and deloitte.</t>
   </si>
 </sst>
 </file>
@@ -1923,27 +1926,51 @@
         <v>76</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
-      <c r="A25" s="13"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="15" t="str">
+    <row r="25" spans="1:14" ht="30.75">
+      <c r="A25" s="13">
+        <v>46265</v>
+      </c>
+      <c r="B25" s="14">
+        <v>560</v>
+      </c>
+      <c r="C25" s="14">
+        <v>20</v>
+      </c>
+      <c r="D25" s="14">
+        <v>60</v>
+      </c>
+      <c r="E25" s="14">
+        <v>60</v>
+      </c>
+      <c r="F25" s="14">
+        <v>300</v>
+      </c>
+      <c r="G25" s="14">
+        <v>6</v>
+      </c>
+      <c r="H25" s="14">
+        <v>20</v>
+      </c>
+      <c r="I25" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="15" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J25" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="17"/>
+        <v>420</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L25" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N25" s="17" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="26" spans="1:14">
       <c r="A26" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 1sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="280" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{402A95FB-9466-4BD5-B9A3-5E0C9D13C9E1}"/>
+  <xr:revisionPtr revIDLastSave="293" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94FF385F-1411-4590-AFAD-35A0189DB041}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="79">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -274,6 +274,9 @@
   </si>
   <si>
     <t>Attended workshop done by google and deloitte.</t>
+  </si>
+  <si>
+    <t>Good day.</t>
   </si>
 </sst>
 </file>
@@ -1972,27 +1975,51 @@
         <v>77</v>
       </c>
     </row>
-    <row r="26" spans="1:14">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15" t="str">
+    <row r="26" spans="1:14" ht="15">
+      <c r="A26" s="13">
+        <v>46266</v>
+      </c>
+      <c r="B26" s="14">
+        <v>520</v>
+      </c>
+      <c r="C26" s="14">
+        <v>20</v>
+      </c>
+      <c r="D26" s="14">
+        <v>60</v>
+      </c>
+      <c r="E26" s="14">
+        <v>120</v>
+      </c>
+      <c r="F26" s="14">
+        <v>300</v>
+      </c>
+      <c r="G26" s="14">
+        <v>6</v>
+      </c>
+      <c r="H26" s="14">
+        <v>0</v>
+      </c>
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="15" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
-      <c r="N26" s="17"/>
+        <v>420</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N26" s="17" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="27" spans="1:14">
       <c r="A27" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 2Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="293" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94FF385F-1411-4590-AFAD-35A0189DB041}"/>
+  <xr:revisionPtr revIDLastSave="305" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EFD629C5-C9AB-4D89-B7FA-556648BA0F3E}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="80">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -277,6 +277,9 @@
   </si>
   <si>
     <t>Good day.</t>
+  </si>
+  <si>
+    <t>Learned new concepts in C++</t>
   </si>
 </sst>
 </file>
@@ -2021,27 +2024,51 @@
         <v>78</v>
       </c>
     </row>
-    <row r="27" spans="1:14">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="15" t="str">
+    <row r="27" spans="1:14" ht="15">
+      <c r="A27" s="13">
+        <v>46267</v>
+      </c>
+      <c r="B27" s="14">
+        <v>570</v>
+      </c>
+      <c r="C27" s="14">
+        <v>20</v>
+      </c>
+      <c r="D27" s="14">
+        <v>120</v>
+      </c>
+      <c r="E27" s="14">
+        <v>60</v>
+      </c>
+      <c r="F27" s="14">
+        <v>300</v>
+      </c>
+      <c r="G27" s="14">
+        <v>6</v>
+      </c>
+      <c r="H27" s="14">
+        <v>0</v>
+      </c>
+      <c r="I27" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
+        <v>1070</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="17"/>
+        <v>370</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N27" s="17" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="28" spans="1:14">
       <c r="A28" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 3Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="305" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EFD629C5-C9AB-4D89-B7FA-556648BA0F3E}"/>
+  <xr:revisionPtr revIDLastSave="328" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92F8BC15-2FA9-4136-9613-355CD36CA16F}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="80">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2070,26 +2070,48 @@
         <v>79</v>
       </c>
     </row>
-    <row r="28" spans="1:14">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+    <row r="28" spans="1:14" ht="15">
+      <c r="A28" s="13">
+        <v>46268</v>
+      </c>
+      <c r="B28" s="14">
+        <v>580</v>
+      </c>
+      <c r="C28" s="14">
+        <v>20</v>
+      </c>
+      <c r="D28" s="14">
+        <v>120</v>
+      </c>
+      <c r="E28" s="14">
+        <v>60</v>
+      </c>
+      <c r="F28" s="14">
+        <v>50</v>
+      </c>
+      <c r="G28" s="14">
+        <v>1</v>
+      </c>
+      <c r="H28" s="14">
+        <v>0</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>830</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
+        <v>610</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>59</v>
+      </c>
       <c r="N28" s="17"/>
     </row>
     <row r="29" spans="1:14">

</xml_diff>

<commit_message>
Daily Activity Tracker 6Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="328" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92F8BC15-2FA9-4136-9613-355CD36CA16F}"/>
+  <xr:revisionPtr revIDLastSave="369" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A7A5D7C-3359-428B-9DF6-CF076F7FBC83}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="84">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -280,6 +280,18 @@
   </si>
   <si>
     <t>Learned new concepts in C++</t>
+  </si>
+  <si>
+    <t>Nice day.</t>
+  </si>
+  <si>
+    <t>Attended session done by HOS.</t>
+  </si>
+  <si>
+    <t>Very good day.</t>
+  </si>
+  <si>
+    <t>Studied for exams.</t>
   </si>
 </sst>
 </file>
@@ -2112,73 +2124,147 @@
       <c r="M28" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="N28" s="17"/>
-    </row>
-    <row r="29" spans="1:14">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+      <c r="N28" s="17" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="15">
+      <c r="A29" s="13">
+        <v>46269</v>
+      </c>
+      <c r="B29" s="14">
+        <v>560</v>
+      </c>
+      <c r="C29" s="14">
+        <v>20</v>
+      </c>
+      <c r="D29" s="14">
+        <v>60</v>
+      </c>
+      <c r="E29" s="14">
+        <v>60</v>
+      </c>
+      <c r="F29" s="14">
+        <v>100</v>
+      </c>
+      <c r="G29" s="14">
+        <v>2</v>
+      </c>
+      <c r="H29" s="14">
+        <v>0</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>800</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="17"/>
-    </row>
-    <row r="30" spans="1:14">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15" t="str">
+        <v>640</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N29" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="15">
+      <c r="A30" s="13">
+        <v>46270</v>
+      </c>
+      <c r="B30" s="14">
+        <v>680</v>
+      </c>
+      <c r="C30" s="14">
+        <v>30</v>
+      </c>
+      <c r="D30" s="14">
+        <v>150</v>
+      </c>
+      <c r="E30" s="14">
+        <v>60</v>
+      </c>
+      <c r="F30" s="14">
+        <v>0</v>
+      </c>
+      <c r="G30" s="14">
+        <v>0</v>
+      </c>
+      <c r="H30" s="14">
+        <v>0</v>
+      </c>
+      <c r="I30" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
+        <v>920</v>
+      </c>
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="17"/>
-    </row>
-    <row r="31" spans="1:14">
-      <c r="A31" s="13"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="15" t="str">
+        <v>520</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="15">
+      <c r="A31" s="13">
+        <v>46271</v>
+      </c>
+      <c r="B31" s="14">
+        <v>620</v>
+      </c>
+      <c r="C31" s="14">
+        <v>20</v>
+      </c>
+      <c r="D31" s="14">
+        <v>180</v>
+      </c>
+      <c r="E31" s="14">
+        <v>120</v>
+      </c>
+      <c r="F31" s="14">
+        <v>0</v>
+      </c>
+      <c r="G31" s="14">
+        <v>0</v>
+      </c>
+      <c r="H31" s="14">
+        <v>0</v>
+      </c>
+      <c r="I31" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
+        <v>940</v>
+      </c>
+      <c r="J31" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="17"/>
+        <v>500</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N31" s="17" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="32" spans="1:14">
       <c r="A32" s="13"/>

</xml_diff>